<commit_message>
fix(template): ship the template with no household data in it
public/phare_template.xlsx carried example figures in its answer columns
(variable budgets ≈ $2,235/mo, annual bills $7,556.18, four goals, and
pre-filled frequencies) that the parser read as the household's own plan.
Every value the parser reads is now cleared; labels, the Example/Notes
columns, formulas, styles and the active sheet are unchanged (edited in the
sheet XML, not re-written).

A prompt row with no amount is no longer counted as an unreadable row, so an
untouched form reports nothing to fix. A test parses the shipped file and
asserts zero income, expense, sinking-fund and goal lines.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/phare_template.xlsx
+++ b/public/phare_template.xlsx
@@ -1128,12 +1128,8 @@
       <c r="A6" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="17">
-        <v>0</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>9</v>
-      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
       <c r="D6" s="16"/>
       <c r="E6" s="14" t="s">
         <v>10</v>
@@ -1143,12 +1139,8 @@
       <c r="A7" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="17">
-        <v>0</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>11</v>
-      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
       <c r="D7" s="16"/>
       <c r="E7" s="14" t="s">
         <v>12</v>
@@ -1158,12 +1150,8 @@
       <c r="A8" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="17">
-        <v>0</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>14</v>
-      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="16"/>
       <c r="E8" s="14" t="s">
         <v>15</v>
@@ -1173,12 +1161,8 @@
       <c r="A9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="17">
-        <v>0</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>14</v>
-      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="16"/>
       <c r="E9" s="14" t="s">
         <v>15</v>
@@ -1239,12 +1223,8 @@
       <c r="B4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
       <c r="E4" s="2" t="s">
         <v>51</v>
       </c>
@@ -1257,12 +1237,8 @@
       <c r="B5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
       <c r="E5" s="3" t="s">
         <v>51</v>
       </c>
@@ -1275,12 +1251,8 @@
       <c r="B6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
       <c r="E6" s="2" t="s">
         <v>51</v>
       </c>
@@ -1293,12 +1265,8 @@
       <c r="B7" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="3" t="s">
         <v>51</v>
       </c>
@@ -1311,12 +1279,8 @@
       <c r="B8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
       <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
@@ -1329,12 +1293,8 @@
       <c r="B9" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="5">
-        <v>0</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="3" t="s">
         <v>51</v>
       </c>
@@ -1347,12 +1307,8 @@
       <c r="B10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
       <c r="E10" s="2" t="s">
         <v>51</v>
       </c>
@@ -1365,12 +1321,8 @@
       <c r="B11" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="5">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="3" t="s">
         <v>51</v>
       </c>
@@ -1383,12 +1335,8 @@
       <c r="B12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="4">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
       <c r="E12" s="2" t="s">
         <v>51</v>
       </c>
@@ -1401,12 +1349,8 @@
       <c r="B13" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C13" s="5">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
       <c r="E13" s="3" t="s">
         <v>51</v>
       </c>
@@ -1419,12 +1363,8 @@
       <c r="B14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="4">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
@@ -1435,12 +1375,8 @@
       <c r="B15" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="5">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="3" t="s">
         <v>117</v>
       </c>
@@ -1453,12 +1389,8 @@
       <c r="B16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="4">
-        <v>0</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
@@ -1469,12 +1401,8 @@
       <c r="B17" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="5">
-        <v>0</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>14</v>
-      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
         <v>69</v>
@@ -1585,12 +1513,8 @@
       <c r="A5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="5">
-        <v>800</v>
-      </c>
-      <c r="C5" s="5">
-        <v>0</v>
-      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
       <c r="D5" s="3" t="s">
         <v>75</v>
       </c>
@@ -1600,12 +1524,8 @@
       <c r="A6" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="4">
-        <v>350</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
       <c r="D6" s="2" t="s">
         <v>75</v>
       </c>
@@ -1615,12 +1535,8 @@
       <c r="A7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="5">
-        <v>50</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
       <c r="D7" s="3" t="s">
         <v>75</v>
       </c>
@@ -1630,12 +1546,8 @@
       <c r="A8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="4">
-        <v>150</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
       <c r="D8" s="2" t="s">
         <v>75</v>
       </c>
@@ -1645,12 +1557,8 @@
       <c r="A9" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="5">
-        <v>335</v>
-      </c>
-      <c r="C9" s="5">
-        <v>0</v>
-      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
       <c r="D9" s="3" t="s">
         <v>75</v>
       </c>
@@ -1660,12 +1568,8 @@
       <c r="A10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="4">
-        <v>100</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="2" t="s">
         <v>75</v>
       </c>
@@ -1675,12 +1579,8 @@
       <c r="A11" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="5">
-        <v>100</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0</v>
-      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
       <c r="D11" s="3" t="s">
         <v>119</v>
       </c>
@@ -1690,12 +1590,8 @@
       <c r="A12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="4">
-        <v>100</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0</v>
-      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
       <c r="D12" s="2" t="s">
         <v>129</v>
       </c>
@@ -1705,12 +1601,8 @@
       <c r="A13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="5">
-        <v>150</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0</v>
-      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
       <c r="D13" s="3" t="s">
         <v>75</v>
       </c>
@@ -1720,12 +1612,8 @@
       <c r="A14" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="4">
-        <v>100</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0</v>
-      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
       <c r="D14" s="2" t="s">
         <v>75</v>
       </c>
@@ -1822,16 +1710,12 @@
       <c r="A6" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="4">
-        <v>3106.18</v>
-      </c>
+      <c r="B6" s="4"/>
       <c r="C6" s="4">
         <f t="shared" ref="C6:C12" si="0">B6/12</f>
-        <v>258.8483333333333</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>91</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
         <v>51</v>
       </c>
@@ -1843,16 +1727,12 @@
       <c r="A7" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="5">
-        <v>350</v>
-      </c>
+      <c r="B7" s="5"/>
       <c r="C7" s="5">
         <f t="shared" si="0"/>
-        <v>29.166666666666668</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
         <v>51</v>
       </c>
@@ -1862,16 +1742,12 @@
       <c r="A8" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="4">
-        <v>2000</v>
-      </c>
+      <c r="B8" s="4"/>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>166.66666666666666</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>96</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
@@ -1883,16 +1759,12 @@
       <c r="A9" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="5">
-        <v>200</v>
-      </c>
+      <c r="B9" s="5"/>
       <c r="C9" s="5">
         <f t="shared" si="0"/>
-        <v>16.666666666666668</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>99</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
         <v>65</v>
       </c>
@@ -1904,16 +1776,12 @@
       <c r="A10" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="4">
-        <v>300</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>102</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
         <v>65</v>
       </c>
@@ -1923,16 +1791,12 @@
       <c r="A11" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="5">
-        <v>600</v>
-      </c>
+      <c r="B11" s="5"/>
       <c r="C11" s="5">
         <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>104</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
         <v>65</v>
       </c>
@@ -1944,16 +1808,12 @@
       <c r="A12" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="4">
-        <v>1000</v>
-      </c>
+      <c r="B12" s="4"/>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>83.333333333333329</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
         <v>51</v>
       </c>
@@ -1981,11 +1841,11 @@
       </c>
       <c r="B15" s="7">
         <f>SUM(B6:B14)</f>
-        <v>7556.18</v>
+        <v>0</v>
       </c>
       <c r="C15" s="7">
         <f>SUM(C6:C14)</f>
-        <v>629.68166666666673</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2034,55 +1894,33 @@
       <c r="A4" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B4" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B5" s="5">
-        <v>8000</v>
-      </c>
-      <c r="C5" s="10">
-        <v>46753</v>
-      </c>
-      <c r="D5" s="5">
-        <v>0</v>
-      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="4">
-        <v>5000</v>
-      </c>
-      <c r="C6" s="11">
-        <v>47115</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="5">
-        <v>5000</v>
-      </c>
+      <c r="B7" s="5"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="5">
-        <v>0</v>
-      </c>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>

</xml_diff>